<commit_message>
farmer product tab completed
</commit_message>
<xml_diff>
--- a/ReportsAndDocuments/worklog.xlsx
+++ b/ReportsAndDocuments/worklog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\300392759\Downloads\working\W26_4495_S3_ManeeshaE\ReportsAndDocuments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4EAF831-5520-46AE-9AAA-29B37518ABAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75BD83EC-5C7C-4B8A-A2D4-F22C214F8E01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="101">
   <si>
     <t>Date</t>
   </si>
@@ -369,6 +369,9 @@
   </si>
   <si>
     <t>sorted issue on updating dispatched items on model submission:solution:demandRequestId id not defined in backend controller farmercontroller.cs</t>
+  </si>
+  <si>
+    <t>created outlet element for nested pages in requireAuth and RequireRole.jsx</t>
   </si>
 </sst>
 </file>
@@ -1053,7 +1056,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DE14CD6-E8F7-4785-AF16-07A58E8D9E8B}">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.28515625" customWidth="1"/>
@@ -1529,6 +1532,11 @@
     <row r="59" spans="1:3">
       <c r="C59" t="s">
         <v>99</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="C60" s="21" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UPDATE vendor dispatches controller
</commit_message>
<xml_diff>
--- a/ReportsAndDocuments/worklog.xlsx
+++ b/ReportsAndDocuments/worklog.xlsx
@@ -5,19 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\300392759\Downloads\working\W26_4495_S3_ManeeshaE\ReportsAndDocuments\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\300392759\Downloads\Dev\W26_4495_S3_ManeeshaE\ReportsAndDocuments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A21FEA08-CB76-4569-BE28-D77B4C429A48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD354402-BD7B-4756-AB91-3FA51FF2EDE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
     <sheet name="Sheet4" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -30,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="115">
   <si>
     <t>Date</t>
   </si>
@@ -405,6 +404,15 @@
   </si>
   <si>
     <t>Completed Farmer Dispatch page frontend + backend (DispatchRowDto.cs, UpdateDispatchStatusDto.cs, FarmerDispatchController.cs, FarmerDispatch.jsx)</t>
+  </si>
+  <si>
+    <t>submitted</t>
+  </si>
+  <si>
+    <t>update vendor dashboard(create dispatch model including filesvendorDashboard.jsx,VendorDemandRequestsController.cs)</t>
+  </si>
+  <si>
+    <t>fully integrated create demand request modal</t>
   </si>
 </sst>
 </file>
@@ -451,18 +459,12 @@
       <name val="Arial Unicode MS"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -717,8 +719,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -731,7 +731,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="16" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -776,60 +776,62 @@
     <xf numFmtId="16" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="16" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="16" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1110,7 +1112,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DE14CD6-E8F7-4785-AF16-07A58E8D9E8B}">
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.28515625" customWidth="1"/>
@@ -1130,20 +1132,20 @@
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="44">
+      <c r="A2" s="47">
         <v>46035</v>
       </c>
-      <c r="B2" s="46">
+      <c r="B2" s="49">
         <v>2</v>
       </c>
-      <c r="C2" s="49" t="s">
+      <c r="C2" s="51" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15.75" thickBot="1">
       <c r="A3" s="48"/>
-      <c r="B3" s="47"/>
-      <c r="C3" s="50"/>
+      <c r="B3" s="50"/>
+      <c r="C3" s="52"/>
     </row>
     <row r="4" spans="1:3" ht="15.75" thickBot="1">
       <c r="A4" s="7"/>
@@ -1210,20 +1212,20 @@
       <c r="C11" s="9"/>
     </row>
     <row r="12" spans="1:3">
-      <c r="A12" s="44">
+      <c r="A12" s="47">
         <v>46039</v>
       </c>
-      <c r="B12" s="46">
+      <c r="B12" s="49">
         <v>2</v>
       </c>
-      <c r="C12" s="49" t="s">
+      <c r="C12" s="51" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="48"/>
-      <c r="B13" s="43"/>
-      <c r="C13" s="51"/>
+      <c r="B13" s="53"/>
+      <c r="C13" s="54"/>
     </row>
     <row r="14" spans="1:3" ht="15.75" thickBot="1">
       <c r="A14" s="7"/>
@@ -1306,10 +1308,10 @@
       </c>
     </row>
     <row r="22" spans="1:3">
-      <c r="A22" s="44">
+      <c r="A22" s="47">
         <v>46049</v>
       </c>
-      <c r="B22" s="46">
+      <c r="B22" s="49">
         <v>3</v>
       </c>
       <c r="C22" s="5" t="s">
@@ -1317,17 +1319,17 @@
       </c>
     </row>
     <row r="23" spans="1:3" ht="15.75" thickBot="1">
-      <c r="A23" s="45"/>
-      <c r="B23" s="47"/>
+      <c r="A23" s="56"/>
+      <c r="B23" s="50"/>
       <c r="C23" s="9" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:3">
-      <c r="A24" s="44">
+      <c r="A24" s="47">
         <v>46051</v>
       </c>
-      <c r="B24" s="46">
+      <c r="B24" s="49">
         <v>4</v>
       </c>
       <c r="C24" s="5" t="s">
@@ -1335,8 +1337,8 @@
       </c>
     </row>
     <row r="25" spans="1:3" ht="15.75" thickBot="1">
-      <c r="A25" s="45"/>
-      <c r="B25" s="47"/>
+      <c r="A25" s="56"/>
+      <c r="B25" s="50"/>
       <c r="C25" s="9" t="s">
         <v>22</v>
       </c>
@@ -1353,10 +1355,10 @@
       </c>
     </row>
     <row r="27" spans="1:3">
-      <c r="A27" s="44">
+      <c r="A27" s="47">
         <v>46057</v>
       </c>
-      <c r="B27" s="46">
+      <c r="B27" s="49">
         <v>3</v>
       </c>
       <c r="C27" s="5" t="s">
@@ -1364,8 +1366,8 @@
       </c>
     </row>
     <row r="28" spans="1:3" ht="15.75" thickBot="1">
-      <c r="A28" s="45"/>
-      <c r="B28" s="47"/>
+      <c r="A28" s="56"/>
+      <c r="B28" s="50"/>
       <c r="C28" s="9" t="s">
         <v>25</v>
       </c>
@@ -1404,29 +1406,29 @@
       </c>
     </row>
     <row r="32" spans="1:3">
-      <c r="A32" s="42"/>
-      <c r="B32" s="43"/>
+      <c r="A32" s="55"/>
+      <c r="B32" s="53"/>
       <c r="C32" s="5" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="33" spans="1:3">
-      <c r="A33" s="42"/>
-      <c r="B33" s="43"/>
+      <c r="A33" s="55"/>
+      <c r="B33" s="53"/>
       <c r="C33" s="5" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="34" spans="1:3">
-      <c r="A34" s="42"/>
-      <c r="B34" s="43"/>
+      <c r="A34" s="55"/>
+      <c r="B34" s="53"/>
       <c r="C34" s="5" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="35" spans="1:3">
-      <c r="A35" s="42"/>
-      <c r="B35" s="43"/>
+      <c r="A35" s="55"/>
+      <c r="B35" s="53"/>
       <c r="C35" s="5" t="s">
         <v>32</v>
       </c>
@@ -1515,102 +1517,115 @@
         <v>44</v>
       </c>
     </row>
-    <row r="49" spans="1:3">
+    <row r="49" spans="1:4">
       <c r="A49" s="17">
         <v>46071</v>
       </c>
-      <c r="C49" s="20" t="s">
+      <c r="C49" s="57" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="50" spans="1:3">
-      <c r="C50" s="21" t="s">
+    <row r="50" spans="1:4">
+      <c r="C50" s="58" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="51" spans="1:3">
-      <c r="C51" s="21" t="s">
+    <row r="51" spans="1:4">
+      <c r="C51" s="58" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="52" spans="1:3">
-      <c r="C52" s="21" t="s">
+    <row r="52" spans="1:4">
+      <c r="C52" s="58" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="53" spans="1:3">
-      <c r="C53" s="21" t="s">
+    <row r="53" spans="1:4">
+      <c r="C53" s="58" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="54" spans="1:3">
+    <row r="54" spans="1:4">
       <c r="A54" s="17">
         <v>46076</v>
       </c>
-      <c r="C54" s="21" t="s">
+      <c r="C54" s="58" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="55" spans="1:3">
+    <row r="55" spans="1:4">
       <c r="A55" s="17">
         <v>46077</v>
       </c>
-      <c r="C55" t="s">
+      <c r="C55" s="58" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="56" spans="1:3">
+    <row r="56" spans="1:4">
       <c r="A56" s="17">
         <v>46081</v>
       </c>
-      <c r="C56" s="21" t="s">
+      <c r="C56" s="58" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="57" spans="1:3">
+    <row r="57" spans="1:4">
       <c r="A57" s="17">
         <v>46082</v>
       </c>
-      <c r="C57" t="s">
+      <c r="C57" s="58" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="58" spans="1:3">
+    <row r="58" spans="1:4">
       <c r="A58" s="17">
         <v>46083</v>
       </c>
-      <c r="C58" s="21" t="s">
+      <c r="C58" s="58" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="59" spans="1:3">
-      <c r="C59" t="s">
+    <row r="59" spans="1:4">
+      <c r="C59" s="58" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="60" spans="1:3">
-      <c r="C60" s="21" t="s">
+    <row r="60" spans="1:4">
+      <c r="C60" s="58" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="61" spans="1:3">
-      <c r="C61" t="s">
+    <row r="61" spans="1:4">
+      <c r="C61" s="58" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="62" spans="1:3">
-      <c r="C62" s="21" t="s">
+    <row r="62" spans="1:4">
+      <c r="C62" s="58" t="s">
         <v>102</v>
+      </c>
+      <c r="D62" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
+      <c r="A63" s="43">
+        <v>46084</v>
+      </c>
+      <c r="B63" s="20"/>
+      <c r="C63" s="20" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
+      <c r="A64" s="20"/>
+      <c r="B64" s="20"/>
+      <c r="C64" s="20" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C12:C13"/>
     <mergeCell ref="A32:A35"/>
     <mergeCell ref="B32:B35"/>
     <mergeCell ref="A22:A23"/>
@@ -1619,6 +1634,12 @@
     <mergeCell ref="B24:B25"/>
     <mergeCell ref="A27:A28"/>
     <mergeCell ref="B27:B28"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -1627,519 +1648,535 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C36D1A51-7B38-4D49-AACB-A85A6A2358FE}">
-  <dimension ref="B2:D58"/>
+  <dimension ref="B2:E60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="7.7109375" style="22" customWidth="1"/>
-    <col min="3" max="3" width="11.85546875" style="22" customWidth="1"/>
-    <col min="4" max="4" width="82.28515625" style="22" customWidth="1"/>
+    <col min="2" max="2" width="7.7109375" style="20" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" style="20" customWidth="1"/>
+    <col min="4" max="4" width="82.28515625" style="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:4">
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="26" t="s">
+      <c r="C2" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="26" t="s">
+      <c r="D2" s="24" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="2:4" ht="30">
-      <c r="B3" s="36">
+      <c r="B3" s="34">
         <v>46035</v>
       </c>
-      <c r="C3" s="29">
+      <c r="C3" s="27">
         <v>2</v>
       </c>
-      <c r="D3" s="28" t="s">
+      <c r="D3" s="26" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="4" spans="2:4">
-      <c r="B4" s="31"/>
-      <c r="C4" s="29">
+      <c r="B4" s="29"/>
+      <c r="C4" s="27">
         <v>1</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="D4" s="26" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="30">
-      <c r="B5" s="40">
+      <c r="B5" s="38">
         <v>46036</v>
       </c>
-      <c r="C5" s="30">
+      <c r="C5" s="28">
         <v>4</v>
       </c>
-      <c r="D5" s="28" t="s">
+      <c r="D5" s="26" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="6" spans="2:4">
-      <c r="B6" s="36">
+      <c r="B6" s="34">
         <v>46037</v>
       </c>
-      <c r="C6" s="30">
+      <c r="C6" s="28">
         <v>4</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="27" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="7" spans="2:4">
-      <c r="B7" s="32"/>
-      <c r="C7" s="32"/>
-      <c r="D7" s="29" t="s">
+      <c r="B7" s="30"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="27" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="8" spans="2:4">
-      <c r="B8" s="32"/>
-      <c r="C8" s="32"/>
-      <c r="D8" s="29" t="s">
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="27" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="9" spans="2:4">
-      <c r="B9" s="32"/>
-      <c r="C9" s="32"/>
-      <c r="D9" s="29" t="s">
+      <c r="B9" s="30"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="27" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="10" spans="2:4">
-      <c r="B10" s="31"/>
-      <c r="C10" s="31"/>
-      <c r="D10" s="29" t="s">
+      <c r="B10" s="29"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="27" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="11" spans="2:4">
-      <c r="B11" s="35">
+      <c r="B11" s="33">
         <v>46039</v>
       </c>
-      <c r="C11" s="31">
+      <c r="C11" s="29">
         <v>2</v>
       </c>
-      <c r="D11" s="28" t="s">
+      <c r="D11" s="26" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="12" spans="2:4">
-      <c r="B12" s="27">
+      <c r="B12" s="25">
         <v>46042</v>
       </c>
-      <c r="C12" s="28">
+      <c r="C12" s="26">
         <v>0.5</v>
       </c>
-      <c r="D12" s="28" t="s">
+      <c r="D12" s="26" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="13" spans="2:4">
-      <c r="B13" s="27">
+      <c r="B13" s="25">
         <v>46043</v>
       </c>
-      <c r="C13" s="28">
+      <c r="C13" s="26">
         <v>2</v>
       </c>
-      <c r="D13" s="28" t="s">
+      <c r="D13" s="26" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="14" spans="2:4">
-      <c r="B14" s="36">
+      <c r="B14" s="34">
         <v>46044</v>
       </c>
-      <c r="C14" s="28">
+      <c r="C14" s="26">
         <v>2</v>
       </c>
-      <c r="D14" s="28" t="s">
+      <c r="D14" s="26" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="15" spans="2:4">
-      <c r="B15" s="36">
+      <c r="B15" s="34">
         <v>46046</v>
       </c>
-      <c r="C15" s="29">
+      <c r="C15" s="27">
         <v>2</v>
       </c>
-      <c r="D15" s="28" t="s">
+      <c r="D15" s="26" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="16" spans="2:4">
-      <c r="B16" s="31"/>
-      <c r="C16" s="29">
+      <c r="B16" s="29"/>
+      <c r="C16" s="27">
         <v>2</v>
       </c>
-      <c r="D16" s="28" t="s">
+      <c r="D16" s="26" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="17" spans="2:4">
-      <c r="B17" s="35">
+      <c r="B17" s="33">
         <v>46047</v>
       </c>
-      <c r="C17" s="28">
+      <c r="C17" s="26">
         <v>2</v>
       </c>
-      <c r="D17" s="28" t="s">
+      <c r="D17" s="26" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="18" spans="2:4">
-      <c r="B18" s="27">
+      <c r="B18" s="25">
         <v>46048</v>
       </c>
-      <c r="C18" s="28">
+      <c r="C18" s="26">
         <v>1</v>
       </c>
-      <c r="D18" s="28" t="s">
+      <c r="D18" s="26" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="19" spans="2:4">
-      <c r="B19" s="36">
+      <c r="B19" s="34">
         <v>46049</v>
       </c>
-      <c r="C19" s="28">
+      <c r="C19" s="26">
         <v>3</v>
       </c>
-      <c r="D19" s="28" t="s">
+      <c r="D19" s="26" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="20" spans="2:4">
-      <c r="B20" s="36">
+      <c r="B20" s="34">
         <v>46051</v>
       </c>
-      <c r="C20" s="29">
+      <c r="C20" s="27">
         <v>4</v>
       </c>
-      <c r="D20" s="28" t="s">
+      <c r="D20" s="26" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="21" spans="2:4">
-      <c r="B21" s="31"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="28" t="s">
+      <c r="B21" s="29"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="26" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="22" spans="2:4">
-      <c r="B22" s="40">
+      <c r="B22" s="38">
         <v>46055</v>
       </c>
-      <c r="C22" s="30">
+      <c r="C22" s="28">
         <v>2</v>
       </c>
-      <c r="D22" s="28" t="s">
+      <c r="D22" s="26" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="23" spans="2:4">
-      <c r="B23" s="36">
+      <c r="B23" s="34">
         <v>46057</v>
       </c>
-      <c r="C23" s="30">
+      <c r="C23" s="28">
         <v>3</v>
       </c>
-      <c r="D23" s="29" t="s">
+      <c r="D23" s="27" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="24" spans="2:4">
-      <c r="B24" s="31"/>
-      <c r="C24" s="31"/>
-      <c r="D24" s="29" t="s">
+      <c r="B24" s="29"/>
+      <c r="C24" s="29"/>
+      <c r="D24" s="27" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="25" spans="2:4">
-      <c r="B25" s="27">
+      <c r="B25" s="25">
         <v>46058</v>
       </c>
-      <c r="C25" s="28">
+      <c r="C25" s="26">
         <v>2</v>
       </c>
-      <c r="D25" s="29" t="s">
+      <c r="D25" s="27" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="26" spans="2:4">
-      <c r="B26" s="36">
+      <c r="B26" s="34">
         <v>46061</v>
       </c>
-      <c r="C26" s="30">
+      <c r="C26" s="28">
         <v>4</v>
       </c>
-      <c r="D26" s="29" t="s">
+      <c r="D26" s="27" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="27" spans="2:4">
-      <c r="B27" s="31"/>
-      <c r="C27" s="31"/>
-      <c r="D27" s="29" t="s">
+      <c r="B27" s="29"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="27" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="28" spans="2:4">
-      <c r="B28" s="36">
+      <c r="B28" s="34">
         <v>46062</v>
       </c>
-      <c r="C28" s="30">
+      <c r="C28" s="28">
         <v>5</v>
       </c>
-      <c r="D28" s="29" t="s">
+      <c r="D28" s="27" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="29" spans="2:4">
-      <c r="B29" s="32"/>
-      <c r="C29" s="32"/>
-      <c r="D29" s="29" t="s">
+      <c r="B29" s="30"/>
+      <c r="C29" s="30"/>
+      <c r="D29" s="27" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="30" spans="2:4">
-      <c r="B30" s="32"/>
-      <c r="C30" s="32"/>
-      <c r="D30" s="29" t="s">
+      <c r="B30" s="30"/>
+      <c r="C30" s="30"/>
+      <c r="D30" s="27" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="31" spans="2:4">
-      <c r="B31" s="31"/>
-      <c r="C31" s="31"/>
-      <c r="D31" s="29" t="s">
+      <c r="B31" s="29"/>
+      <c r="C31" s="29"/>
+      <c r="D31" s="27" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="32" spans="2:4">
-      <c r="B32" s="36">
+      <c r="B32" s="34">
         <v>46063</v>
       </c>
-      <c r="C32" s="30">
+      <c r="C32" s="28">
         <v>5</v>
       </c>
-      <c r="D32" s="29" t="s">
+      <c r="D32" s="27" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="33" spans="2:4">
-      <c r="B33" s="31"/>
-      <c r="C33" s="31"/>
-      <c r="D33" s="29" t="s">
+      <c r="B33" s="29"/>
+      <c r="C33" s="29"/>
+      <c r="D33" s="27" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="34" spans="2:4">
-      <c r="B34" s="36">
+      <c r="B34" s="34">
         <v>46065</v>
       </c>
-      <c r="C34" s="30">
+      <c r="C34" s="28">
         <v>4</v>
       </c>
-      <c r="D34" s="29" t="s">
+      <c r="D34" s="27" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="35" spans="2:4">
-      <c r="B35" s="31"/>
-      <c r="C35" s="31"/>
-      <c r="D35" s="29" t="s">
+      <c r="B35" s="29"/>
+      <c r="C35" s="29"/>
+      <c r="D35" s="27" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="36" spans="2:4">
-      <c r="B36" s="36">
+      <c r="B36" s="34">
         <v>46068</v>
       </c>
-      <c r="C36" s="30">
+      <c r="C36" s="28">
         <v>5</v>
       </c>
-      <c r="D36" s="29" t="s">
+      <c r="D36" s="27" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="37" spans="2:4">
-      <c r="B37" s="31"/>
-      <c r="C37" s="31"/>
-      <c r="D37" s="29" t="s">
+      <c r="B37" s="29"/>
+      <c r="C37" s="29"/>
+      <c r="D37" s="27" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="38" spans="2:4">
-      <c r="B38" s="40">
+      <c r="B38" s="38">
         <v>46070</v>
       </c>
-      <c r="C38" s="23">
+      <c r="C38" s="21">
         <v>6</v>
       </c>
-      <c r="D38" s="29" t="s">
+      <c r="D38" s="27" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="39" spans="2:4" ht="30">
-      <c r="B39" s="32"/>
-      <c r="C39" s="23"/>
-      <c r="D39" s="29" t="s">
+      <c r="B39" s="30"/>
+      <c r="C39" s="21"/>
+      <c r="D39" s="27" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="40" spans="2:4">
-      <c r="B40" s="32"/>
-      <c r="C40" s="23"/>
-      <c r="D40" s="29" t="s">
+      <c r="B40" s="30"/>
+      <c r="C40" s="21"/>
+      <c r="D40" s="27" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="41" spans="2:4">
-      <c r="B41" s="32"/>
-      <c r="C41" s="23"/>
-      <c r="D41" s="29" t="s">
+      <c r="B41" s="30"/>
+      <c r="C41" s="21"/>
+      <c r="D41" s="27" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="42" spans="2:4">
-      <c r="B42" s="32"/>
-      <c r="C42" s="23"/>
-      <c r="D42" s="29" t="s">
+      <c r="B42" s="30"/>
+      <c r="C42" s="21"/>
+      <c r="D42" s="27" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="43" spans="2:4">
-      <c r="B43" s="32"/>
-      <c r="C43" s="23"/>
-      <c r="D43" s="29" t="s">
+      <c r="B43" s="30"/>
+      <c r="C43" s="21"/>
+      <c r="D43" s="27" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="44" spans="2:4">
-      <c r="B44" s="31"/>
-      <c r="C44" s="34"/>
-      <c r="D44" s="29" t="s">
+      <c r="B44" s="29"/>
+      <c r="C44" s="32"/>
+      <c r="D44" s="27" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="45" spans="2:4" ht="30">
-      <c r="B45" s="40">
+      <c r="B45" s="38">
         <v>46071</v>
       </c>
-      <c r="C45" s="32">
+      <c r="C45" s="30">
         <v>6</v>
       </c>
-      <c r="D45" s="28" t="s">
+      <c r="D45" s="26" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="46" spans="2:4">
-      <c r="B46" s="36">
+      <c r="B46" s="34">
         <v>46076</v>
       </c>
-      <c r="C46" s="33">
+      <c r="C46" s="31">
         <v>8</v>
       </c>
-      <c r="D46" s="29" t="s">
+      <c r="D46" s="27" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="47" spans="2:4" ht="30">
-      <c r="B47" s="32"/>
-      <c r="C47" s="23"/>
-      <c r="D47" s="29" t="s">
+      <c r="B47" s="30"/>
+      <c r="C47" s="21"/>
+      <c r="D47" s="27" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="48" spans="2:4">
-      <c r="B48" s="38"/>
-      <c r="C48" s="24"/>
-      <c r="D48" s="37" t="s">
+      <c r="B48" s="36"/>
+      <c r="C48" s="22"/>
+      <c r="D48" s="35" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="49" spans="2:4">
-      <c r="B49" s="39"/>
-      <c r="C49" s="25"/>
-      <c r="D49" s="37" t="s">
+    <row r="49" spans="2:5">
+      <c r="B49" s="37"/>
+      <c r="C49" s="23"/>
+      <c r="D49" s="35" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="50" spans="2:4" ht="30">
-      <c r="B50" s="52">
+    <row r="50" spans="2:5" ht="30">
+      <c r="B50" s="40">
         <v>46077</v>
       </c>
-      <c r="C50" s="53"/>
-      <c r="D50" s="54" t="s">
+      <c r="C50" s="41"/>
+      <c r="D50" s="42" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="51" spans="2:4" ht="30">
-      <c r="B51" s="52">
+    <row r="51" spans="2:5" ht="30">
+      <c r="B51" s="40">
         <v>46081</v>
       </c>
-      <c r="C51" s="53"/>
-      <c r="D51" s="54" t="s">
+      <c r="C51" s="41"/>
+      <c r="D51" s="42" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="52" spans="2:4">
-      <c r="B52" s="52">
+    <row r="52" spans="2:5">
+      <c r="B52" s="40">
         <v>46082</v>
       </c>
-      <c r="C52" s="53"/>
-      <c r="D52" s="54" t="s">
+      <c r="C52" s="41"/>
+      <c r="D52" s="42" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="53" spans="2:4" ht="30">
-      <c r="B53" s="55">
+    <row r="53" spans="2:5" ht="30">
+      <c r="B53" s="43">
         <v>46083</v>
       </c>
-      <c r="C53" s="58"/>
-      <c r="D53" s="54" t="s">
+      <c r="C53" s="46"/>
+      <c r="D53" s="42" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="54" spans="2:4" ht="30">
-      <c r="B54" s="56"/>
-      <c r="C54" s="56"/>
-      <c r="D54" s="54" t="s">
+    <row r="54" spans="2:5" ht="30">
+      <c r="B54" s="44"/>
+      <c r="C54" s="44"/>
+      <c r="D54" s="42" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="55" spans="2:4" ht="30">
-      <c r="B55" s="56"/>
-      <c r="C55" s="56"/>
-      <c r="D55" s="54" t="s">
+    <row r="55" spans="2:5" ht="30">
+      <c r="B55" s="44"/>
+      <c r="C55" s="44"/>
+      <c r="D55" s="42" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="56" spans="2:4" ht="45">
-      <c r="B56" s="56"/>
-      <c r="C56" s="56"/>
-      <c r="D56" s="54" t="s">
+    <row r="56" spans="2:5" ht="45">
+      <c r="B56" s="44"/>
+      <c r="C56" s="44"/>
+      <c r="D56" s="42" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="57" spans="2:4" ht="30">
-      <c r="B57" s="56"/>
-      <c r="C57" s="56"/>
-      <c r="D57" s="54" t="s">
+    <row r="57" spans="2:5" ht="30">
+      <c r="B57" s="44"/>
+      <c r="C57" s="44"/>
+      <c r="D57" s="42" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="58" spans="2:4" ht="30">
-      <c r="B58" s="57"/>
-      <c r="C58" s="57"/>
-      <c r="D58" s="54" t="s">
+    <row r="58" spans="2:5" ht="30">
+      <c r="B58" s="45"/>
+      <c r="C58" s="45"/>
+      <c r="D58" s="42" t="s">
         <v>111</v>
+      </c>
+      <c r="E58" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="59" spans="2:5">
+      <c r="B59" s="43">
+        <v>46084</v>
+      </c>
+      <c r="D59" s="20" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="60" spans="2:5">
+      <c r="D60" s="20" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update worklog -10th March
</commit_message>
<xml_diff>
--- a/ReportsAndDocuments/worklog.xlsx
+++ b/ReportsAndDocuments/worklog.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\300392759\Desktop\dev\W26_4495_S3_ManeeshaE\ReportsAndDocuments\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\300392759\Downloads\dev\W26_4495_S3_ManeeshaE\ReportsAndDocuments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDFEA4A9-0AB6-48EA-8DDC-E7CEFF7F6E48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C72A2D5-AE24-4371-BA78-103EFD2C69BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="184">
   <si>
     <t>Date</t>
   </si>
@@ -893,6 +893,12 @@
   </si>
   <si>
     <t xml:space="preserve">March 3–9 </t>
+  </si>
+  <si>
+    <t>individual checking</t>
+  </si>
+  <si>
+    <t>changing research baseline model to ML related model which focus on ML.NET’s forecasting task -provide more in detail</t>
   </si>
 </sst>
 </file>
@@ -1219,7 +1225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1370,92 +1376,95 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="8" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="16" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="8" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1757,20 +1766,20 @@
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="56">
+      <c r="A2" s="73">
         <v>46035</v>
       </c>
-      <c r="B2" s="58">
+      <c r="B2" s="75">
         <v>2</v>
       </c>
-      <c r="C2" s="61" t="s">
+      <c r="C2" s="77" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15.75" thickBot="1">
-      <c r="A3" s="60"/>
-      <c r="B3" s="59"/>
-      <c r="C3" s="62"/>
+      <c r="A3" s="74"/>
+      <c r="B3" s="76"/>
+      <c r="C3" s="78"/>
     </row>
     <row r="4" spans="1:3" ht="15.75" thickBot="1">
       <c r="A4" s="7"/>
@@ -1837,20 +1846,20 @@
       <c r="C11" s="9"/>
     </row>
     <row r="12" spans="1:3">
-      <c r="A12" s="56">
+      <c r="A12" s="73">
         <v>46039</v>
       </c>
-      <c r="B12" s="58">
+      <c r="B12" s="75">
         <v>2</v>
       </c>
-      <c r="C12" s="61" t="s">
+      <c r="C12" s="77" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:3">
-      <c r="A13" s="60"/>
-      <c r="B13" s="55"/>
-      <c r="C13" s="63"/>
+      <c r="A13" s="74"/>
+      <c r="B13" s="79"/>
+      <c r="C13" s="80"/>
     </row>
     <row r="14" spans="1:3" ht="15.75" thickBot="1">
       <c r="A14" s="7"/>
@@ -1933,10 +1942,10 @@
       </c>
     </row>
     <row r="22" spans="1:3">
-      <c r="A22" s="56">
+      <c r="A22" s="73">
         <v>46049</v>
       </c>
-      <c r="B22" s="58">
+      <c r="B22" s="75">
         <v>3</v>
       </c>
       <c r="C22" s="5" t="s">
@@ -1944,17 +1953,17 @@
       </c>
     </row>
     <row r="23" spans="1:3" ht="15.75" thickBot="1">
-      <c r="A23" s="57"/>
-      <c r="B23" s="59"/>
+      <c r="A23" s="82"/>
+      <c r="B23" s="76"/>
       <c r="C23" s="9" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:3">
-      <c r="A24" s="56">
+      <c r="A24" s="73">
         <v>46051</v>
       </c>
-      <c r="B24" s="58">
+      <c r="B24" s="75">
         <v>4</v>
       </c>
       <c r="C24" s="5" t="s">
@@ -1962,8 +1971,8 @@
       </c>
     </row>
     <row r="25" spans="1:3" ht="15.75" thickBot="1">
-      <c r="A25" s="57"/>
-      <c r="B25" s="59"/>
+      <c r="A25" s="82"/>
+      <c r="B25" s="76"/>
       <c r="C25" s="9" t="s">
         <v>22</v>
       </c>
@@ -1980,10 +1989,10 @@
       </c>
     </row>
     <row r="27" spans="1:3">
-      <c r="A27" s="56">
+      <c r="A27" s="73">
         <v>46057</v>
       </c>
-      <c r="B27" s="58">
+      <c r="B27" s="75">
         <v>3</v>
       </c>
       <c r="C27" s="5" t="s">
@@ -1991,8 +2000,8 @@
       </c>
     </row>
     <row r="28" spans="1:3" ht="15.75" thickBot="1">
-      <c r="A28" s="57"/>
-      <c r="B28" s="59"/>
+      <c r="A28" s="82"/>
+      <c r="B28" s="76"/>
       <c r="C28" s="9" t="s">
         <v>25</v>
       </c>
@@ -2031,29 +2040,29 @@
       </c>
     </row>
     <row r="32" spans="1:3">
-      <c r="A32" s="54"/>
-      <c r="B32" s="55"/>
+      <c r="A32" s="81"/>
+      <c r="B32" s="79"/>
       <c r="C32" s="5" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="33" spans="1:3">
-      <c r="A33" s="54"/>
-      <c r="B33" s="55"/>
+      <c r="A33" s="81"/>
+      <c r="B33" s="79"/>
       <c r="C33" s="5" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="34" spans="1:3">
-      <c r="A34" s="54"/>
-      <c r="B34" s="55"/>
+      <c r="A34" s="81"/>
+      <c r="B34" s="79"/>
       <c r="C34" s="5" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="35" spans="1:3">
-      <c r="A35" s="54"/>
-      <c r="B35" s="55"/>
+      <c r="A35" s="81"/>
+      <c r="B35" s="79"/>
       <c r="C35" s="5" t="s">
         <v>32</v>
       </c>
@@ -2251,12 +2260,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C12:C13"/>
     <mergeCell ref="A32:A35"/>
     <mergeCell ref="B32:B35"/>
     <mergeCell ref="A22:A23"/>
@@ -2265,6 +2268,12 @@
     <mergeCell ref="B24:B25"/>
     <mergeCell ref="A27:A28"/>
     <mergeCell ref="B27:B28"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -2885,7 +2894,7 @@
       </c>
     </row>
     <row r="74" spans="2:4">
-      <c r="B74" s="64">
+      <c r="B74" s="54">
         <v>46089</v>
       </c>
       <c r="D74" s="20" t="s">
@@ -2893,7 +2902,7 @@
       </c>
     </row>
     <row r="75" spans="2:4">
-      <c r="B75" s="64">
+      <c r="B75" s="54">
         <v>46090</v>
       </c>
       <c r="D75" s="20" t="s">
@@ -2931,63 +2940,63 @@
       </c>
     </row>
     <row r="83" spans="4:4">
-      <c r="D83" s="65"/>
+      <c r="D83" s="55"/>
     </row>
     <row r="84" spans="4:4">
-      <c r="D84" s="66" t="s">
+      <c r="D84" s="56" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="85" spans="4:4">
-      <c r="D85" s="65"/>
+      <c r="D85" s="55"/>
     </row>
     <row r="86" spans="4:4">
-      <c r="D86" s="66" t="s">
+      <c r="D86" s="56" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="87" spans="4:4">
-      <c r="D87" s="65"/>
+      <c r="D87" s="55"/>
     </row>
     <row r="88" spans="4:4">
-      <c r="D88" s="66" t="s">
+      <c r="D88" s="56" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="89" spans="4:4">
-      <c r="D89" s="65"/>
+      <c r="D89" s="55"/>
     </row>
     <row r="90" spans="4:4">
-      <c r="D90" s="66" t="s">
+      <c r="D90" s="56" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="91" spans="4:4">
-      <c r="D91" s="65"/>
+      <c r="D91" s="55"/>
     </row>
     <row r="92" spans="4:4">
-      <c r="D92" s="65" t="s">
+      <c r="D92" s="55" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="93" spans="4:4">
-      <c r="D93" s="65"/>
+      <c r="D93" s="55"/>
     </row>
     <row r="94" spans="4:4">
-      <c r="D94" s="68" t="s">
+      <c r="D94" s="58" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="95" spans="4:4">
-      <c r="D95" s="67"/>
+      <c r="D95" s="57"/>
     </row>
     <row r="96" spans="4:4">
-      <c r="D96" s="67" t="s">
+      <c r="D96" s="57" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="100" spans="4:4" ht="180">
-      <c r="D100" s="69" t="s">
+      <c r="D100" s="59" t="s">
         <v>144</v>
       </c>
     </row>
@@ -2999,7 +3008,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE4CB711-9D7B-4FAA-801C-2959CA58D8D4}">
-  <dimension ref="B2:D23"/>
+  <dimension ref="B2:D25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="11.7109375" customWidth="1"/>
@@ -3008,21 +3017,21 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:4">
-      <c r="B2" s="77" t="s">
+      <c r="B2" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="78" t="s">
+      <c r="C2" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="77" t="s">
+      <c r="D2" s="67" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B3" s="76">
+      <c r="B3" s="66">
         <v>46084</v>
       </c>
-      <c r="C3" s="70">
+      <c r="C3" s="60">
         <v>6</v>
       </c>
       <c r="D3" s="41" t="s">
@@ -3030,24 +3039,24 @@
       </c>
     </row>
     <row r="4" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B4" s="74"/>
-      <c r="C4" s="71"/>
+      <c r="B4" s="64"/>
+      <c r="C4" s="61"/>
       <c r="D4" s="41" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B5" s="75"/>
-      <c r="C5" s="72"/>
+      <c r="B5" s="65"/>
+      <c r="C5" s="62"/>
       <c r="D5" s="41" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B6" s="76">
+      <c r="B6" s="66">
         <v>46086</v>
       </c>
-      <c r="C6" s="73">
+      <c r="C6" s="63">
         <v>5</v>
       </c>
       <c r="D6" s="41" t="s">
@@ -3055,24 +3064,24 @@
       </c>
     </row>
     <row r="7" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B7" s="74"/>
-      <c r="C7" s="74"/>
+      <c r="B7" s="64"/>
+      <c r="C7" s="64"/>
       <c r="D7" s="41" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="8" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B8" s="75"/>
-      <c r="C8" s="75"/>
+      <c r="B8" s="65"/>
+      <c r="C8" s="65"/>
       <c r="D8" s="41" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B9" s="76">
+      <c r="B9" s="66">
         <v>46088</v>
       </c>
-      <c r="C9" s="73">
+      <c r="C9" s="63">
         <v>6</v>
       </c>
       <c r="D9" s="41" t="s">
@@ -3080,45 +3089,45 @@
       </c>
     </row>
     <row r="10" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B10" s="74"/>
-      <c r="C10" s="74"/>
+      <c r="B10" s="64"/>
+      <c r="C10" s="64"/>
       <c r="D10" s="41" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B11" s="74"/>
-      <c r="C11" s="74"/>
+      <c r="B11" s="64"/>
+      <c r="C11" s="64"/>
       <c r="D11" s="41" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="12" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B12" s="74"/>
-      <c r="C12" s="74"/>
+      <c r="B12" s="64"/>
+      <c r="C12" s="64"/>
       <c r="D12" s="41" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B13" s="74"/>
-      <c r="C13" s="74"/>
+      <c r="B13" s="64"/>
+      <c r="C13" s="64"/>
       <c r="D13" s="41" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B14" s="75"/>
-      <c r="C14" s="75"/>
+      <c r="B14" s="65"/>
+      <c r="C14" s="65"/>
       <c r="D14" s="41" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B15" s="76">
+      <c r="B15" s="66">
         <v>46089</v>
       </c>
-      <c r="C15" s="73">
+      <c r="C15" s="63">
         <v>3</v>
       </c>
       <c r="D15" s="41" t="s">
@@ -3126,17 +3135,17 @@
       </c>
     </row>
     <row r="16" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B16" s="75"/>
-      <c r="C16" s="75"/>
+      <c r="B16" s="65"/>
+      <c r="C16" s="65"/>
       <c r="D16" s="41" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B17" s="76">
+      <c r="B17" s="66">
         <v>46090</v>
       </c>
-      <c r="C17" s="73">
+      <c r="C17" s="63">
         <v>6</v>
       </c>
       <c r="D17" s="41" t="s">
@@ -3144,45 +3153,61 @@
       </c>
     </row>
     <row r="18" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B18" s="74"/>
-      <c r="C18" s="74"/>
+      <c r="B18" s="64"/>
+      <c r="C18" s="64"/>
       <c r="D18" s="41" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B19" s="74"/>
-      <c r="C19" s="74"/>
+      <c r="B19" s="64"/>
+      <c r="C19" s="64"/>
       <c r="D19" s="41" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="20" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B20" s="74"/>
-      <c r="C20" s="74"/>
+      <c r="B20" s="64"/>
+      <c r="C20" s="64"/>
       <c r="D20" s="41" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="21" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B21" s="74"/>
-      <c r="C21" s="74"/>
+      <c r="B21" s="64"/>
+      <c r="C21" s="64"/>
       <c r="D21" s="41" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="22" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B22" s="74"/>
-      <c r="C22" s="74"/>
+      <c r="B22" s="64"/>
+      <c r="C22" s="64"/>
       <c r="D22" s="41" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="23" spans="2:4" ht="38.25" customHeight="1">
-      <c r="B23" s="75"/>
-      <c r="C23" s="75"/>
+      <c r="B23" s="65"/>
+      <c r="C23" s="65"/>
       <c r="D23" s="41" t="s">
         <v>165</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4">
+      <c r="B24" s="17">
+        <v>46091</v>
+      </c>
+      <c r="C24">
+        <v>6</v>
+      </c>
+      <c r="D24" s="83" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" ht="30">
+      <c r="D25" s="83" t="s">
+        <v>183</v>
       </c>
     </row>
   </sheetData>
@@ -3193,7 +3218,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F000D01-920E-4EFE-A851-9564F79E29F6}">
-  <dimension ref="B1:D8"/>
+  <dimension ref="B1:D9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="13.28515625" customWidth="1"/>
@@ -3204,80 +3229,85 @@
   <sheetData>
     <row r="1" spans="2:4" ht="15.75" thickBot="1"/>
     <row r="2" spans="2:4" ht="17.25" thickBot="1">
-      <c r="B2" s="82" t="s">
+      <c r="B2" s="72" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="82" t="s">
+      <c r="C2" s="72" t="s">
         <v>166</v>
       </c>
-      <c r="D2" s="82" t="s">
+      <c r="D2" s="72" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="3" spans="2:4" ht="231.75" thickBot="1">
-      <c r="B3" s="79">
+      <c r="B3" s="69">
         <v>46084</v>
       </c>
-      <c r="C3" s="80" t="s">
+      <c r="C3" s="70" t="s">
         <v>168</v>
       </c>
-      <c r="D3" s="80" t="s">
+      <c r="D3" s="70" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="4" spans="2:4" ht="99.75" thickBot="1">
-      <c r="B4" s="79">
+      <c r="B4" s="69">
         <v>46088</v>
       </c>
-      <c r="C4" s="80" t="s">
+      <c r="C4" s="70" t="s">
         <v>170</v>
       </c>
-      <c r="D4" s="80" t="s">
+      <c r="D4" s="70" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="149.25" thickBot="1">
-      <c r="B5" s="81" t="s">
+      <c r="B5" s="71" t="s">
         <v>172</v>
       </c>
-      <c r="C5" s="80" t="s">
+      <c r="C5" s="70" t="s">
         <v>173</v>
       </c>
-      <c r="D5" s="80" t="s">
+      <c r="D5" s="70" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="116.25" thickBot="1">
-      <c r="B6" s="79">
+      <c r="B6" s="69">
         <v>46089</v>
       </c>
-      <c r="C6" s="80" t="s">
+      <c r="C6" s="70" t="s">
         <v>175</v>
       </c>
-      <c r="D6" s="80" t="s">
+      <c r="D6" s="70" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="182.25" thickBot="1">
-      <c r="B7" s="79">
+      <c r="B7" s="69">
         <v>46090</v>
       </c>
-      <c r="C7" s="80" t="s">
+      <c r="C7" s="70" t="s">
         <v>177</v>
       </c>
-      <c r="D7" s="80" t="s">
+      <c r="D7" s="70" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="8" spans="2:4" ht="132.75" thickBot="1">
-      <c r="B8" s="81" t="s">
+      <c r="B8" s="71" t="s">
         <v>181</v>
       </c>
-      <c r="C8" s="80" t="s">
+      <c r="C8" s="70" t="s">
         <v>179</v>
       </c>
-      <c r="D8" s="80" t="s">
+      <c r="D8" s="70" t="s">
         <v>180</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4">
+      <c r="B9" s="17">
+        <v>46091</v>
       </c>
     </row>
   </sheetData>

</xml_diff>